<commit_message>
Self learning variable ,tab space ,new line
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -495,22 +495,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>300</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>uuu</t>
+          <t>Ohid</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>iii</t>
+          <t>EEE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>3.00</t>
         </is>
       </c>
     </row>

</xml_diff>